<commit_message>
docs!: remove empty page ASVS_5.0_Tracker
</commit_message>
<xml_diff>
--- a/Deliverables/asvs-assessment/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/asvs-assessment/ASVS_5.0_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diogomartins/Documents/Universidade/Mestrado/1º ano/2º semestre/DESOFS/desofs2026-thu_crr_1/Deliverables/asvs-assessment/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FAF7EEFD-9558-1A4F-99DD-751C9BD56225}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EED25457-81C5-F94A-A4AB-B8DF198CF5CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="500" firstSheet="10" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="500" firstSheet="11" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>

</xml_diff>